<commit_message>
remove oversized installer from repository
</commit_message>
<xml_diff>
--- a/Module/MainModel/整车CAN20260630_MB分配.xlsx
+++ b/Module/MainModel/整车CAN20260630_MB分配.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12280" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12280" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="MB分配说明_更新" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5355" uniqueCount="979">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5371" uniqueCount="979">
   <si>
     <r>
       <rPr>
@@ -5744,7 +5744,9 @@
       <c r="D15" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E15" s="3"/>
+      <c r="E15" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F15" s="3" t="s">
         <v>19</v>
       </c>
@@ -5780,7 +5782,9 @@
       <c r="D16" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="E16" s="3"/>
+      <c r="E16" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F16" s="3" t="s">
         <v>19</v>
       </c>
@@ -5816,7 +5820,9 @@
       <c r="D17" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F17" s="3" t="s">
         <v>19</v>
       </c>
@@ -5852,7 +5858,9 @@
       <c r="D18" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="E18" s="3"/>
+      <c r="E18" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F18" s="3" t="s">
         <v>122</v>
       </c>
@@ -5888,7 +5896,9 @@
       <c r="D19" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F19" s="3" t="s">
         <v>94</v>
       </c>
@@ -5924,7 +5934,9 @@
       <c r="D20" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F20" s="3" t="s">
         <v>129</v>
       </c>
@@ -5960,7 +5972,9 @@
       <c r="D21" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E21" s="3"/>
+      <c r="E21" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F21" s="3" t="s">
         <v>19</v>
       </c>
@@ -5996,7 +6010,9 @@
       <c r="D22" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E22" s="3"/>
+      <c r="E22" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F22" s="3" t="s">
         <v>94</v>
       </c>
@@ -6032,7 +6048,9 @@
       <c r="D23" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F23" s="3" t="s">
         <v>129</v>
       </c>
@@ -6068,7 +6086,9 @@
       <c r="D24" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="3"/>
+      <c r="E24" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F24" s="3" t="s">
         <v>19</v>
       </c>
@@ -6104,7 +6124,9 @@
       <c r="D25" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="E25" s="3"/>
+      <c r="E25" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F25" s="3" t="s">
         <v>19</v>
       </c>
@@ -6292,7 +6314,9 @@
       <c r="D30" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="E30" s="3"/>
+      <c r="E30" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F30" s="3" t="s">
         <v>19</v>
       </c>
@@ -6328,7 +6352,9 @@
       <c r="D31" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E31" s="3"/>
+      <c r="E31" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F31" s="3" t="s">
         <v>19</v>
       </c>
@@ -6364,7 +6390,9 @@
       <c r="D32" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E32" s="3"/>
+      <c r="E32" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F32" s="3" t="s">
         <v>94</v>
       </c>
@@ -6400,7 +6428,9 @@
       <c r="D33" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E33" s="3"/>
+      <c r="E33" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F33" s="3" t="s">
         <v>94</v>
       </c>
@@ -6436,7 +6466,9 @@
       <c r="D34" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E34" s="3"/>
+      <c r="E34" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="F34" s="3" t="s">
         <v>19</v>
       </c>

</xml_diff>